<commit_message>
Ajout des extensions pharm manquantes 7ad614333e45ab2c9c290c28bfd7ea6d07d4090d
</commit_message>
<xml_diff>
--- a/enrichissement-pharm/ig/StructureDefinition-fr-cda-antecedents-familiaux.xlsx
+++ b/enrichissement-pharm/ig/StructureDefinition-fr-cda-antecedents-familiaux.xlsx
@@ -45,7 +45,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>CDA - FR Antecedents familiaux</t>
+    <t>CDA - FR Entrée Antecedents familiaux</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-29T09:37:21+00:00</t>
+    <t>2026-08-03T10:14:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>